<commit_message>
Measurements at 325Mhz and 300Mhz. Implementation Pictures of Floorplan for both architectures
</commit_message>
<xml_diff>
--- a/results/GEMV_Area_Comparison.xlsx
+++ b/results/GEMV_Area_Comparison.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Area" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="System" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -54,7 +55,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -127,6 +133,8 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1282,4 +1290,509 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>System-level area - the whole accelerator on the device</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>POST-ROUTE, IN-SYSTEM, from the Vitis link's report_accelerator_utilization. Unlike the Area sheet, this INCLUDES the HLS data movers (17 CUs sparse, 14 dense) and the platform shell. Both builds are 300 MHz: sparse with the SLR floorplan, dense without -- which is what each design was actually measured on. Never mix these numbers with the OOC ones on the Area sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1. WHERE THE LOGIC IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Sparse LUT</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Dense LUT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Sparse cost</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>vs dense</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>engine (gemv CU)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>66167</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46926</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>19241</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.4100285555981759</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>the compute engine as placed IN SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>movers: mm2s</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>20690</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>15365</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>5325</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.3465668727627725</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>13 read movers vs 10 -- the 3 extra carry the sparsity INDICES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>movers: s2mm</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>8139</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>8135</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0.0004917025199754148</v>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>4 write movers in both -- the output path is unchanged by sparsity</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ALL user logic</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>94996</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>70426</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>24570</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.3488768352597052</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>everything inside the dynamic region</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>platform (shell)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>123821</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>118929</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>4892</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0.04113378570407554</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>not ours -- grows only because more HBM channels are wired up</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>THE MOVERS ARE NOT A ROUNDING ERROR. Sparse: 66,167 LUTs of engine plus 28,829 of movers = 94,996 of user logic, so the data movers are 30% of the accelerator (dense: 33%). An area claim that quotes only the engine understates the real cost by about a third. Both numbers belong in the thesis, labelled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>THE ENGINE DELTA AGREES WITH THE OOC MEASUREMENT: +41.0%% in system against +41.1%% out-of-context. Two independent implementations -- different tool context, different constraint, different clock target -- landing within 0.1 point. That is the area result cross-validated, and it is worth saying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>The absolute engine figure does move: 66,167 LUTs in system against 62,417 OOC, +6.0%, because the engine is re-optimised in context with the platform. So the two sheets are not interchangeable even though their DELTAS agree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2. FULL RESOURCE PICTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>LUT</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>LUTAsMem</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>BRAM</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>SPARSE</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr"/>
+      <c r="C18" s="20" t="inlineStr"/>
+      <c r="D18" s="20" t="inlineStr"/>
+      <c r="E18" s="20" t="inlineStr"/>
+      <c r="F18" s="20" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>krnl_gemv_sparse</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>66167</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>5758</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>87238</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>krnl_mm2s</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>20690</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>3549</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>36720</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>176</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>krnl_s2mm</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>8139</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>3672</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>12692</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Used Resources</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>94996</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>12979</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>136650</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>314</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>123821</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>15703</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>191830</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>204</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>DENSE</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr"/>
+      <c r="C24" s="20" t="inlineStr"/>
+      <c r="D24" s="20" t="inlineStr"/>
+      <c r="E24" s="20" t="inlineStr"/>
+      <c r="F24" s="20" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>krnl_gemv_dense</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>46926</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>5760</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>79432</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>krnl_mm2s</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>15365</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>2730</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>28955</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>krnl_s2mm</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>8135</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>3672</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>12691</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Used Resources</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>70426</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>12162</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>121078</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>268</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>118929</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>14458</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>182598</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>202</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A12:F12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>